<commit_message>
new localizer files with better spread of same exemplars and localizer font size and image size adusted
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/retrieval_block1_fixed-middle-10_00.xlsx
+++ b/psychopy_exp_files/sequences/retrieval_block1_fixed-middle-10_00.xlsx
@@ -567,12 +567,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -654,12 +654,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -723,12 +723,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -810,12 +810,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -879,12 +879,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -966,12 +966,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1035,12 +1035,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1122,12 +1122,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1434,12 +1434,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1503,12 +1503,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1659,12 +1659,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1746,12 +1746,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1902,12 +1902,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -2058,12 +2058,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -2127,12 +2127,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -2214,12 +2214,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -2283,12 +2283,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -2370,12 +2370,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -2439,12 +2439,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -2526,12 +2526,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -2595,12 +2595,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -2751,12 +2751,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -2838,12 +2838,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -2907,12 +2907,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -2994,12 +2994,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -3063,12 +3063,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -3150,12 +3150,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -3219,12 +3219,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -3375,12 +3375,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -3462,12 +3462,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -3531,12 +3531,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -3618,12 +3618,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -3687,12 +3687,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -3774,12 +3774,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -3843,12 +3843,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -3930,12 +3930,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -3999,12 +3999,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -4086,12 +4086,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -4242,12 +4242,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -4311,12 +4311,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr"/>
@@ -4398,12 +4398,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -4467,12 +4467,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
@@ -4554,12 +4554,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -4623,12 +4623,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -4710,12 +4710,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -4779,12 +4779,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
@@ -4866,12 +4866,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -4935,12 +4935,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
@@ -5022,12 +5022,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -5091,12 +5091,12 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
@@ -5178,12 +5178,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -5247,12 +5247,12 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
@@ -5334,12 +5334,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
@@ -5403,12 +5403,12 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
@@ -5490,12 +5490,12 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
@@ -5559,12 +5559,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
@@ -5646,12 +5646,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -5715,12 +5715,12 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
@@ -5802,12 +5802,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -5871,12 +5871,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
@@ -5958,12 +5958,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -6027,12 +6027,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
@@ -6114,12 +6114,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
@@ -6183,12 +6183,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -6270,12 +6270,12 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -6339,12 +6339,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
@@ -6426,12 +6426,12 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -6495,12 +6495,12 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
@@ -6582,12 +6582,12 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -6651,12 +6651,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H80" t="inlineStr"/>
@@ -6738,12 +6738,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H81" t="inlineStr"/>
@@ -6807,12 +6807,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
@@ -6894,12 +6894,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
@@ -6963,12 +6963,12 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
@@ -7050,12 +7050,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
@@ -7119,12 +7119,12 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
@@ -7206,12 +7206,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
@@ -7275,12 +7275,12 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
@@ -7362,12 +7362,12 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
@@ -7431,12 +7431,12 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
@@ -7518,12 +7518,12 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
@@ -7587,12 +7587,12 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
@@ -7674,12 +7674,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
@@ -7743,12 +7743,12 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
@@ -7830,12 +7830,12 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
@@ -7899,12 +7899,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H96" t="inlineStr"/>
@@ -7986,12 +7986,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H97" t="inlineStr"/>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H98" t="inlineStr"/>
@@ -8142,12 +8142,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H99" t="inlineStr"/>
@@ -8211,12 +8211,12 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H100" t="inlineStr"/>
@@ -8298,12 +8298,12 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
@@ -8367,12 +8367,12 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H102" t="inlineStr"/>
@@ -8454,12 +8454,12 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
@@ -8523,12 +8523,12 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H104" t="inlineStr"/>
@@ -8610,12 +8610,12 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
@@ -8679,12 +8679,12 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H106" t="inlineStr"/>
@@ -8766,12 +8766,12 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H107" t="inlineStr"/>
@@ -8835,12 +8835,12 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
@@ -8922,12 +8922,12 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
@@ -8991,12 +8991,12 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
@@ -9078,12 +9078,12 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H111" t="inlineStr"/>
@@ -9147,12 +9147,12 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H112" t="inlineStr"/>
@@ -9234,12 +9234,12 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
@@ -9303,12 +9303,12 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H114" t="inlineStr"/>
@@ -9390,12 +9390,12 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H115" t="inlineStr"/>
@@ -9459,12 +9459,12 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H116" t="inlineStr"/>
@@ -9546,12 +9546,12 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
@@ -9615,12 +9615,12 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -9702,12 +9702,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -9771,12 +9771,12 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H120" t="inlineStr"/>
@@ -9858,12 +9858,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -9927,12 +9927,12 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -10014,12 +10014,12 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H123" t="inlineStr"/>
@@ -10083,12 +10083,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H124" t="inlineStr"/>
@@ -10170,12 +10170,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H125" t="inlineStr"/>
@@ -10239,12 +10239,12 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H126" t="inlineStr"/>
@@ -10326,12 +10326,12 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H127" t="inlineStr"/>
@@ -10395,12 +10395,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H128" t="inlineStr"/>
@@ -10482,12 +10482,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
@@ -10551,12 +10551,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
@@ -10638,12 +10638,12 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
@@ -10707,12 +10707,12 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H132" t="inlineStr"/>
@@ -10794,12 +10794,12 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H133" t="inlineStr"/>
@@ -10863,12 +10863,12 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
@@ -10950,12 +10950,12 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H135" t="inlineStr"/>
@@ -11019,12 +11019,12 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H136" t="inlineStr"/>
@@ -11106,12 +11106,12 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H137" t="inlineStr"/>
@@ -11175,12 +11175,12 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H138" t="inlineStr"/>
@@ -11262,12 +11262,12 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
@@ -11331,12 +11331,12 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H140" t="inlineStr"/>
@@ -11418,12 +11418,12 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H141" t="inlineStr"/>
@@ -11487,12 +11487,12 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H142" t="inlineStr"/>
@@ -11574,12 +11574,12 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H143" t="inlineStr"/>
@@ -11643,12 +11643,12 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H144" t="inlineStr"/>
@@ -11730,12 +11730,12 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H145" t="inlineStr"/>
@@ -11799,12 +11799,12 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H146" t="inlineStr"/>
@@ -11886,12 +11886,12 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H147" t="inlineStr"/>
@@ -11955,12 +11955,12 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H148" t="inlineStr"/>
@@ -12042,12 +12042,12 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H149" t="inlineStr"/>
@@ -12111,12 +12111,12 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H150" t="inlineStr"/>
@@ -12198,12 +12198,12 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H151" t="inlineStr"/>
@@ -12267,12 +12267,12 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H152" t="inlineStr"/>
@@ -12354,12 +12354,12 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H153" t="inlineStr"/>
@@ -12423,12 +12423,12 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H154" t="inlineStr"/>
@@ -12510,12 +12510,12 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H155" t="inlineStr"/>
@@ -12579,12 +12579,12 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H156" t="inlineStr"/>
@@ -12666,12 +12666,12 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H157" t="inlineStr"/>
@@ -12735,12 +12735,12 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H158" t="inlineStr"/>
@@ -12822,12 +12822,12 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="H159" t="inlineStr"/>
@@ -12891,12 +12891,12 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H160" t="inlineStr"/>
@@ -12978,12 +12978,12 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H161" t="inlineStr"/>
@@ -13047,12 +13047,12 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H162" t="inlineStr"/>
@@ -13134,12 +13134,12 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H163" t="inlineStr"/>
@@ -13203,12 +13203,12 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H164" t="inlineStr"/>
@@ -13290,12 +13290,12 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H165" t="inlineStr"/>
@@ -13359,12 +13359,12 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H166" t="inlineStr"/>
@@ -13446,12 +13446,12 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="H167" t="inlineStr"/>
@@ -13515,12 +13515,12 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H168" t="inlineStr"/>
@@ -13602,12 +13602,12 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H169" t="inlineStr"/>
@@ -13671,12 +13671,12 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H170" t="inlineStr"/>
@@ -13758,12 +13758,12 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H171" t="inlineStr"/>
@@ -13827,12 +13827,12 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H172" t="inlineStr"/>
@@ -13914,12 +13914,12 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H173" t="inlineStr"/>
@@ -13983,12 +13983,12 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H174" t="inlineStr"/>
@@ -14070,12 +14070,12 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H175" t="inlineStr"/>
@@ -14139,12 +14139,12 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H176" t="inlineStr"/>
@@ -14226,12 +14226,12 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H177" t="inlineStr"/>
@@ -14295,12 +14295,12 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H178" t="inlineStr"/>
@@ -14382,12 +14382,12 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H179" t="inlineStr"/>
@@ -14451,12 +14451,12 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H180" t="inlineStr"/>
@@ -14538,12 +14538,12 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H181" t="inlineStr"/>
@@ -14607,12 +14607,12 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H182" t="inlineStr"/>
@@ -14694,12 +14694,12 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H183" t="inlineStr"/>
@@ -14763,12 +14763,12 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H184" t="inlineStr"/>
@@ -14850,12 +14850,12 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H185" t="inlineStr"/>
@@ -14919,12 +14919,12 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H186" t="inlineStr"/>
@@ -15006,12 +15006,12 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H187" t="inlineStr"/>
@@ -15075,12 +15075,12 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H188" t="inlineStr"/>
@@ -15162,12 +15162,12 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H189" t="inlineStr"/>
@@ -15231,12 +15231,12 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H190" t="inlineStr"/>
@@ -15318,12 +15318,12 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H191" t="inlineStr"/>
@@ -15387,12 +15387,12 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H192" t="inlineStr"/>
@@ -15474,12 +15474,12 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H193" t="inlineStr"/>
@@ -15543,12 +15543,12 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H194" t="inlineStr"/>
@@ -15630,12 +15630,12 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H195" t="inlineStr"/>
@@ -15699,12 +15699,12 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H196" t="inlineStr"/>
@@ -15786,12 +15786,12 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H197" t="inlineStr"/>
@@ -15855,12 +15855,12 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H198" t="inlineStr"/>
@@ -15942,12 +15942,12 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H199" t="inlineStr"/>
@@ -16011,12 +16011,12 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H200" t="inlineStr"/>
@@ -16098,12 +16098,12 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H201" t="inlineStr"/>
@@ -16167,12 +16167,12 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H202" t="inlineStr"/>
@@ -16254,12 +16254,12 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H203" t="inlineStr"/>
@@ -16323,12 +16323,12 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H204" t="inlineStr"/>
@@ -16410,12 +16410,12 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H205" t="inlineStr"/>
@@ -16479,12 +16479,12 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H206" t="inlineStr"/>
@@ -16566,12 +16566,12 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H207" t="inlineStr"/>
@@ -16635,12 +16635,12 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H208" t="inlineStr"/>
@@ -16722,12 +16722,12 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H209" t="inlineStr"/>
@@ -16791,12 +16791,12 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H210" t="inlineStr"/>
@@ -16878,12 +16878,12 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H211" t="inlineStr"/>
@@ -16947,12 +16947,12 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H212" t="inlineStr"/>
@@ -17034,12 +17034,12 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="H213" t="inlineStr"/>
@@ -17103,12 +17103,12 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H214" t="inlineStr"/>
@@ -17190,12 +17190,12 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H215" t="inlineStr"/>
@@ -17259,12 +17259,12 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H216" t="inlineStr"/>
@@ -17346,12 +17346,12 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H217" t="inlineStr"/>
@@ -17415,12 +17415,12 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H218" t="inlineStr"/>
@@ -17502,12 +17502,12 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H219" t="inlineStr"/>
@@ -17571,12 +17571,12 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H220" t="inlineStr"/>
@@ -17658,12 +17658,12 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="H221" t="inlineStr"/>
@@ -17727,12 +17727,12 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H222" t="inlineStr"/>
@@ -17814,12 +17814,12 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H223" t="inlineStr"/>
@@ -17883,12 +17883,12 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H224" t="inlineStr"/>
@@ -17970,12 +17970,12 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H225" t="inlineStr"/>
@@ -18039,12 +18039,12 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H226" t="inlineStr"/>
@@ -18126,12 +18126,12 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H227" t="inlineStr"/>
@@ -18195,12 +18195,12 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H228" t="inlineStr"/>
@@ -18282,12 +18282,12 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H229" t="inlineStr"/>
@@ -18351,12 +18351,12 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H230" t="inlineStr"/>
@@ -18438,12 +18438,12 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>stimuli/house/house_30.jpg</t>
+          <t>stimuli/house/house_25.jpg</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="H231" t="inlineStr"/>
@@ -18507,12 +18507,12 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H232" t="inlineStr"/>
@@ -18594,12 +18594,12 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_07.jpg</t>
+          <t>stimuli/flower/flower_05.jpg</t>
         </is>
       </c>
       <c r="H233" t="inlineStr"/>
@@ -18663,12 +18663,12 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H234" t="inlineStr"/>
@@ -18750,12 +18750,12 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_49.jpg</t>
+          <t>stimuli/bicycle/bicycle_13.jpg</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_37.jpg</t>
+          <t>stimuli/ball/ball_40.jpg</t>
         </is>
       </c>
       <c r="H235" t="inlineStr"/>
@@ -18819,12 +18819,12 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H236" t="inlineStr"/>
@@ -18906,12 +18906,12 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_38.jpg</t>
+          <t>stimuli/hand/hand_12.jpg</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_29.jpg</t>
+          <t>stimuli/jacket/jacket_07.jpg</t>
         </is>
       </c>
       <c r="H237" t="inlineStr"/>
@@ -18975,12 +18975,12 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H238" t="inlineStr"/>
@@ -19062,12 +19062,12 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_21.jpg</t>
+          <t>stimuli/chair/chair_25.jpg</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_35.jpg</t>
+          <t>stimuli/hammer/hammer_09.jpg</t>
         </is>
       </c>
       <c r="H239" t="inlineStr"/>
@@ -19131,12 +19131,12 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H240" t="inlineStr"/>
@@ -19218,12 +19218,12 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_04.jpg</t>
+          <t>stimuli/bread/bread_09.jpg</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_36.jpg</t>
+          <t>stimuli/dog/dog_39.jpg</t>
         </is>
       </c>
       <c r="H241" t="inlineStr"/>

</xml_diff>